<commit_message>
mdb and rddt updates
</commit_message>
<xml_diff>
--- a/MDB.xlsx
+++ b/MDB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeffe\Documents\GitHub\martinshkreli-models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B41A1735-D2B9-484F-B635-DC603A79CD80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2A6420E-818E-4DBB-AA5D-CCA58FA4EA51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3870" yWindow="105" windowWidth="26190" windowHeight="20805" activeTab="1" xr2:uid="{9A102858-C73E-5D48-A2CD-E1A822063168}"/>
+    <workbookView xWindow="40305" yWindow="90" windowWidth="11310" windowHeight="20805" activeTab="1" xr2:uid="{9A102858-C73E-5D48-A2CD-E1A822063168}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -506,7 +506,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -552,6 +552,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1630,20 +1633,18 @@
         <v>518</v>
       </c>
       <c r="O16" s="4">
-        <f>+N16+26</f>
-        <v>544</v>
+        <v>549.01400000000001</v>
       </c>
       <c r="P16" s="4">
-        <f>+O16+26</f>
-        <v>570</v>
+        <v>591.40200000000004</v>
       </c>
       <c r="Q16" s="4">
         <f>+P16+26</f>
-        <v>596</v>
+        <v>617.40200000000004</v>
       </c>
       <c r="R16" s="4">
         <f>+Q16+26</f>
-        <v>622</v>
+        <v>643.40200000000004</v>
       </c>
       <c r="U16" s="4">
         <v>873.78200000000004</v>
@@ -1661,215 +1662,215 @@
       </c>
       <c r="Y16" s="13">
         <f>SUM(O16:R16)</f>
-        <v>2332</v>
+        <v>2401.2200000000003</v>
       </c>
       <c r="Z16" s="4">
         <f>+Y16*(1+$AC$36)</f>
-        <v>2798.4</v>
+        <v>2881.4640000000004</v>
       </c>
       <c r="AA16" s="4">
         <f t="shared" ref="AA16:AG16" si="1">+Z16*(1+$AC$36)</f>
-        <v>3358.08</v>
+        <v>3457.7568000000006</v>
       </c>
       <c r="AB16" s="4">
         <f t="shared" si="1"/>
-        <v>4029.6959999999999</v>
+        <v>4149.3081600000005</v>
       </c>
       <c r="AC16" s="4">
         <f t="shared" si="1"/>
-        <v>4835.6351999999997</v>
+        <v>4979.1697920000006</v>
       </c>
       <c r="AD16" s="4">
         <f t="shared" si="1"/>
-        <v>5802.7622399999991</v>
+        <v>5975.0037504000002</v>
       </c>
       <c r="AE16" s="4">
         <f t="shared" si="1"/>
-        <v>6963.3146879999986</v>
+        <v>7170.0045004800004</v>
       </c>
       <c r="AF16" s="4">
         <f t="shared" si="1"/>
-        <v>8355.9776255999986</v>
+        <v>8604.0054005759994</v>
       </c>
       <c r="AG16" s="4">
         <f t="shared" si="1"/>
-        <v>10027.173150719998</v>
+        <v>10324.806480691199</v>
       </c>
       <c r="AH16" s="4">
         <f>AG16*(1+$AC$37)</f>
-        <v>10127.444882227199</v>
+        <v>10428.054545498111</v>
       </c>
       <c r="AI16" s="4">
         <f t="shared" ref="AI16:BY16" si="2">AH16*(1+$AC$37)</f>
-        <v>10228.719331049471</v>
+        <v>10532.335090953093</v>
       </c>
       <c r="AJ16" s="4">
         <f t="shared" si="2"/>
-        <v>10331.006524359966</v>
+        <v>10637.658441862624</v>
       </c>
       <c r="AK16" s="4">
         <f t="shared" si="2"/>
-        <v>10434.316589603566</v>
+        <v>10744.03502628125</v>
       </c>
       <c r="AL16" s="4">
         <f t="shared" si="2"/>
-        <v>10538.659755499602</v>
+        <v>10851.475376544062</v>
       </c>
       <c r="AM16" s="4">
         <f t="shared" si="2"/>
-        <v>10644.046353054599</v>
+        <v>10959.990130309503</v>
       </c>
       <c r="AN16" s="4">
         <f t="shared" si="2"/>
-        <v>10750.486816585144</v>
+        <v>11069.590031612599</v>
       </c>
       <c r="AO16" s="4">
         <f t="shared" si="2"/>
-        <v>10857.991684750996</v>
+        <v>11180.285931928725</v>
       </c>
       <c r="AP16" s="4">
         <f t="shared" si="2"/>
-        <v>10966.571601598505</v>
+        <v>11292.088791248012</v>
       </c>
       <c r="AQ16" s="4">
         <f t="shared" si="2"/>
-        <v>11076.23731761449</v>
+        <v>11405.009679160492</v>
       </c>
       <c r="AR16" s="4">
         <f t="shared" si="2"/>
-        <v>11186.999690790635</v>
+        <v>11519.059775952097</v>
       </c>
       <c r="AS16" s="4">
         <f t="shared" si="2"/>
-        <v>11298.869687698541</v>
+        <v>11634.250373711619</v>
       </c>
       <c r="AT16" s="4">
         <f t="shared" si="2"/>
-        <v>11411.858384575527</v>
+        <v>11750.592877448735</v>
       </c>
       <c r="AU16" s="4">
         <f t="shared" si="2"/>
-        <v>11525.976968421282</v>
+        <v>11868.098806223223</v>
       </c>
       <c r="AV16" s="4">
         <f t="shared" si="2"/>
-        <v>11641.236738105496</v>
+        <v>11986.779794285456</v>
       </c>
       <c r="AW16" s="4">
         <f t="shared" si="2"/>
-        <v>11757.649105486551</v>
+        <v>12106.64759222831</v>
       </c>
       <c r="AX16" s="4">
         <f t="shared" si="2"/>
-        <v>11875.225596541417</v>
+        <v>12227.714068150593</v>
       </c>
       <c r="AY16" s="4">
         <f t="shared" si="2"/>
-        <v>11993.97785250683</v>
+        <v>12349.9912088321</v>
       </c>
       <c r="AZ16" s="4">
         <f t="shared" si="2"/>
-        <v>12113.917631031898</v>
+        <v>12473.49112092042</v>
       </c>
       <c r="BA16" s="4">
         <f t="shared" si="2"/>
-        <v>12235.056807342216</v>
+        <v>12598.226032129625</v>
       </c>
       <c r="BB16" s="4">
         <f t="shared" si="2"/>
-        <v>12357.407375415638</v>
+        <v>12724.208292450921</v>
       </c>
       <c r="BC16" s="4">
         <f t="shared" si="2"/>
-        <v>12480.981449169794</v>
+        <v>12851.450375375431</v>
       </c>
       <c r="BD16" s="4">
         <f t="shared" si="2"/>
-        <v>12605.791263661493</v>
+        <v>12979.964879129186</v>
       </c>
       <c r="BE16" s="4">
         <f t="shared" si="2"/>
-        <v>12731.849176298108</v>
+        <v>13109.764527920477</v>
       </c>
       <c r="BF16" s="4">
         <f t="shared" si="2"/>
-        <v>12859.167668061089</v>
+        <v>13240.862173199683</v>
       </c>
       <c r="BG16" s="4">
         <f t="shared" si="2"/>
-        <v>12987.7593447417</v>
+        <v>13373.270794931679</v>
       </c>
       <c r="BH16" s="4">
         <f t="shared" si="2"/>
-        <v>13117.636938189118</v>
+        <v>13507.003502880996</v>
       </c>
       <c r="BI16" s="4">
         <f t="shared" si="2"/>
-        <v>13248.81330757101</v>
+        <v>13642.073537909806</v>
       </c>
       <c r="BJ16" s="4">
         <f t="shared" si="2"/>
-        <v>13381.301440646721</v>
+        <v>13778.494273288905</v>
       </c>
       <c r="BK16" s="4">
         <f t="shared" si="2"/>
-        <v>13515.114455053188</v>
+        <v>13916.279216021794</v>
       </c>
       <c r="BL16" s="4">
         <f t="shared" si="2"/>
-        <v>13650.265599603719</v>
+        <v>14055.442008182012</v>
       </c>
       <c r="BM16" s="4">
         <f t="shared" si="2"/>
-        <v>13786.768255599756</v>
+        <v>14195.996428263832</v>
       </c>
       <c r="BN16" s="4">
         <f t="shared" si="2"/>
-        <v>13924.635938155754</v>
+        <v>14337.95639254647</v>
       </c>
       <c r="BO16" s="4">
         <f t="shared" si="2"/>
-        <v>14063.882297537311</v>
+        <v>14481.335956471934</v>
       </c>
       <c r="BP16" s="4">
         <f t="shared" si="2"/>
-        <v>14204.521120512685</v>
+        <v>14626.149316036654</v>
       </c>
       <c r="BQ16" s="4">
         <f t="shared" si="2"/>
-        <v>14346.566331717811</v>
+        <v>14772.410809197021</v>
       </c>
       <c r="BR16" s="4">
         <f t="shared" si="2"/>
-        <v>14490.031995034989</v>
+        <v>14920.134917288991</v>
       </c>
       <c r="BS16" s="4">
         <f t="shared" si="2"/>
-        <v>14634.932314985339</v>
+        <v>15069.336266461882</v>
       </c>
       <c r="BT16" s="4">
         <f t="shared" si="2"/>
-        <v>14781.281638135193</v>
+        <v>15220.0296291265</v>
       </c>
       <c r="BU16" s="4">
         <f t="shared" si="2"/>
-        <v>14929.094454516546</v>
+        <v>15372.229925417765</v>
       </c>
       <c r="BV16" s="4">
         <f t="shared" si="2"/>
-        <v>15078.385399061712</v>
+        <v>15525.952224671943</v>
       </c>
       <c r="BW16" s="4">
         <f t="shared" si="2"/>
-        <v>15229.169253052329</v>
+        <v>15681.211746918661</v>
       </c>
       <c r="BX16" s="4">
         <f t="shared" si="2"/>
-        <v>15381.460945582852</v>
+        <v>15838.023864387847</v>
       </c>
       <c r="BY16" s="4">
         <f t="shared" si="2"/>
-        <v>15535.275555038681</v>
+        <v>15996.404103031726</v>
       </c>
     </row>
     <row r="17" spans="2:27" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -1914,20 +1915,19 @@
         <v>134.68</v>
       </c>
       <c r="O17" s="10">
-        <f t="shared" si="3"/>
-        <v>141.44</v>
+        <v>158.041</v>
       </c>
       <c r="P17" s="10">
-        <f t="shared" si="3"/>
-        <v>148.19999999999999</v>
+        <f>139.949+31.479</f>
+        <v>171.428</v>
       </c>
       <c r="Q17" s="10">
         <f t="shared" si="3"/>
-        <v>154.95999999999998</v>
+        <v>160.52452</v>
       </c>
       <c r="R17" s="10">
         <f>+R16-R18</f>
-        <v>161.72000000000003</v>
+        <v>167.28452000000004</v>
       </c>
       <c r="U17" s="3">
         <f>217.901+41.591</f>
@@ -1947,15 +1947,15 @@
       </c>
       <c r="Y17" s="10">
         <f>SUM(O17:R17)</f>
-        <v>606.31999999999994</v>
+        <v>657.27804000000003</v>
       </c>
       <c r="Z17" s="3">
         <f>+Z16-Z18</f>
-        <v>699.59999999999991</v>
+        <v>720.36599999999999</v>
       </c>
       <c r="AA17" s="3">
         <f>+AA16-AA18</f>
-        <v>839.52</v>
+        <v>864.43920000000026</v>
       </c>
     </row>
     <row r="18" spans="2:27" x14ac:dyDescent="0.2">
@@ -2011,20 +2011,20 @@
         <v>383.32</v>
       </c>
       <c r="O18" s="10">
-        <f>+O16*0.74</f>
-        <v>402.56</v>
+        <f>O16-O17</f>
+        <v>390.97300000000001</v>
       </c>
       <c r="P18" s="10">
-        <f>+P16*0.74</f>
-        <v>421.8</v>
+        <f>P16-P17</f>
+        <v>419.97400000000005</v>
       </c>
       <c r="Q18" s="10">
         <f>+Q16*0.74</f>
-        <v>441.04</v>
+        <v>456.87748000000005</v>
       </c>
       <c r="R18" s="10">
         <f>+R16*0.74</f>
-        <v>460.28</v>
+        <v>476.11748</v>
       </c>
       <c r="U18" s="3">
         <f>+U16-U17</f>
@@ -2044,15 +2044,15 @@
       </c>
       <c r="Y18" s="10">
         <f>+Y16-Y17</f>
-        <v>1725.68</v>
+        <v>1743.9419600000001</v>
       </c>
       <c r="Z18" s="3">
         <f>+Z16*0.75</f>
-        <v>2098.8000000000002</v>
+        <v>2161.0980000000004</v>
       </c>
       <c r="AA18" s="3">
         <f>+AA16*0.75</f>
-        <v>2518.56</v>
+        <v>2593.3176000000003</v>
       </c>
     </row>
     <row r="19" spans="2:27" x14ac:dyDescent="0.2">
@@ -2095,19 +2095,17 @@
         <v>221.67180000000002</v>
       </c>
       <c r="O19" s="10">
-        <f t="shared" ref="O19:O21" si="5">+K19*1.05</f>
-        <v>230.4162</v>
+        <v>220.923</v>
       </c>
       <c r="P19" s="10">
-        <f t="shared" ref="P19:P21" si="6">+L19*1.05</f>
-        <v>232.61595</v>
+        <v>244.065</v>
       </c>
       <c r="Q19" s="10">
-        <f t="shared" ref="Q19:Q21" si="7">+M19*1.05</f>
+        <f t="shared" ref="Q19:Q21" si="5">+M19*1.05</f>
         <v>228.85170000000002</v>
       </c>
       <c r="R19" s="10">
-        <f t="shared" ref="R19:R21" si="8">+N19*1.05</f>
+        <f t="shared" ref="R19:R21" si="6">+N19*1.05</f>
         <v>232.75539000000003</v>
       </c>
       <c r="U19" s="3">
@@ -2117,24 +2115,24 @@
         <v>699.20100000000002</v>
       </c>
       <c r="W19" s="3">
-        <f t="shared" ref="W19:W21" si="9">SUM(G19:J19)</f>
+        <f t="shared" ref="W19:W21" si="7">SUM(G19:J19)</f>
         <v>782.76</v>
       </c>
       <c r="X19" s="10">
-        <f t="shared" ref="X19:X21" si="10">SUM(K19:N19)</f>
+        <f t="shared" ref="X19:X21" si="8">SUM(K19:N19)</f>
         <v>880.60879999999997</v>
       </c>
       <c r="Y19" s="10">
-        <f t="shared" ref="Y19:Y21" si="11">SUM(O19:R19)</f>
-        <v>924.63924000000009</v>
+        <f t="shared" ref="Y19:Y21" si="9">SUM(O19:R19)</f>
+        <v>926.59509000000003</v>
       </c>
       <c r="Z19" s="3">
         <f>+Y19*1.05</f>
-        <v>970.87120200000015</v>
+        <v>972.92484450000006</v>
       </c>
       <c r="AA19" s="3">
         <f>+Z19*1.05</f>
-        <v>1019.4147621000002</v>
+        <v>1021.5710867250001</v>
       </c>
     </row>
     <row r="20" spans="2:27" x14ac:dyDescent="0.2">
@@ -2173,23 +2171,21 @@
         <v>151.41</v>
       </c>
       <c r="N20" s="10">
-        <f t="shared" ref="N20:N21" si="12">+J20*1.05</f>
+        <f t="shared" ref="N20:N21" si="10">+J20*1.05</f>
         <v>152.83064999999999</v>
       </c>
       <c r="O20" s="10">
+        <v>168.82900000000001</v>
+      </c>
+      <c r="P20" s="10">
+        <v>181.739</v>
+      </c>
+      <c r="Q20" s="10">
         <f t="shared" si="5"/>
-        <v>153.363</v>
-      </c>
-      <c r="P20" s="10">
+        <v>158.98050000000001</v>
+      </c>
+      <c r="R20" s="10">
         <f t="shared" si="6"/>
-        <v>156.41535000000002</v>
-      </c>
-      <c r="Q20" s="10">
-        <f t="shared" si="7"/>
-        <v>158.98050000000001</v>
-      </c>
-      <c r="R20" s="10">
-        <f t="shared" si="8"/>
         <v>160.4721825</v>
       </c>
       <c r="U20" s="3">
@@ -2199,24 +2195,24 @@
         <v>421.69200000000001</v>
       </c>
       <c r="W20" s="3">
+        <f t="shared" si="7"/>
+        <v>515.94000000000005</v>
+      </c>
+      <c r="X20" s="10">
+        <f t="shared" si="8"/>
+        <v>599.26765</v>
+      </c>
+      <c r="Y20" s="10">
         <f t="shared" si="9"/>
-        <v>515.94000000000005</v>
-      </c>
-      <c r="X20" s="10">
-        <f t="shared" si="10"/>
-        <v>599.26765</v>
-      </c>
-      <c r="Y20" s="10">
+        <v>670.02068250000002</v>
+      </c>
+      <c r="Z20" s="3">
+        <f t="shared" ref="Z20:AA20" si="11">+Y20*1.05</f>
+        <v>703.52171662500007</v>
+      </c>
+      <c r="AA20" s="3">
         <f t="shared" si="11"/>
-        <v>629.23103250000008</v>
-      </c>
-      <c r="Z20" s="3">
-        <f t="shared" ref="Z20:AA20" si="13">+Y20*1.05</f>
-        <v>660.69258412500017</v>
-      </c>
-      <c r="AA20" s="3">
-        <f t="shared" si="13"/>
-        <v>693.72721333125025</v>
+        <v>738.69780245625009</v>
       </c>
     </row>
     <row r="21" spans="2:27" x14ac:dyDescent="0.2">
@@ -2255,23 +2251,21 @@
         <v>52.555999999999997</v>
       </c>
       <c r="N21" s="10">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>60.540900000000001</v>
       </c>
       <c r="O21" s="10">
+        <v>54.774999999999999</v>
+      </c>
+      <c r="P21" s="10">
+        <v>59.463999999999999</v>
+      </c>
+      <c r="Q21" s="10">
         <f t="shared" si="5"/>
-        <v>63.573300000000003</v>
-      </c>
-      <c r="P21" s="10">
+        <v>55.183799999999998</v>
+      </c>
+      <c r="R21" s="10">
         <f t="shared" si="6"/>
-        <v>53.329500000000003</v>
-      </c>
-      <c r="Q21" s="10">
-        <f t="shared" si="7"/>
-        <v>55.183799999999998</v>
-      </c>
-      <c r="R21" s="10">
-        <f t="shared" si="8"/>
         <v>63.567945000000002</v>
       </c>
       <c r="U21" s="3">
@@ -2281,24 +2275,24 @@
         <v>160.49799999999999</v>
       </c>
       <c r="W21" s="3">
+        <f t="shared" si="7"/>
+        <v>193.55799999999999</v>
+      </c>
+      <c r="X21" s="10">
+        <f t="shared" si="8"/>
+        <v>224.43289999999999</v>
+      </c>
+      <c r="Y21" s="10">
         <f t="shared" si="9"/>
-        <v>193.55799999999999</v>
-      </c>
-      <c r="X21" s="10">
-        <f t="shared" si="10"/>
-        <v>224.43289999999999</v>
-      </c>
-      <c r="Y21" s="10">
-        <f t="shared" si="11"/>
-        <v>235.65454500000001</v>
+        <v>232.990745</v>
       </c>
       <c r="Z21" s="3">
-        <f t="shared" ref="Z21:AA21" si="14">+Y21*1.05</f>
-        <v>247.43727225000004</v>
+        <f t="shared" ref="Z21:AA21" si="12">+Y21*1.05</f>
+        <v>244.64028225000001</v>
       </c>
       <c r="AA21" s="3">
-        <f t="shared" si="14"/>
-        <v>259.80913586250006</v>
+        <f t="shared" si="12"/>
+        <v>256.87229636250004</v>
       </c>
     </row>
     <row r="22" spans="2:27" x14ac:dyDescent="0.2">
@@ -2306,96 +2300,96 @@
         <v>35</v>
       </c>
       <c r="C22" s="3">
-        <f t="shared" ref="C22:N22" si="15">SUM(C19:C21)</f>
+        <f t="shared" ref="C22:N22" si="13">SUM(C19:C21)</f>
         <v>0</v>
       </c>
       <c r="D22" s="3">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>330.226</v>
       </c>
       <c r="E22" s="3">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>322.89200000000005</v>
       </c>
       <c r="F22" s="3">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>345.101</v>
       </c>
       <c r="G22" s="3">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>339.37800000000004</v>
       </c>
       <c r="H22" s="3">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>367.45699999999999</v>
       </c>
       <c r="I22" s="3">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>371.096</v>
       </c>
       <c r="J22" s="3">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>414.327</v>
       </c>
       <c r="K22" s="3">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>426.05</v>
       </c>
       <c r="L22" s="3">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>421.29599999999999</v>
       </c>
       <c r="M22" s="3">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>421.92</v>
       </c>
       <c r="N22" s="3">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>435.04335000000003</v>
       </c>
       <c r="O22" s="3">
-        <f t="shared" ref="O22:R22" si="16">SUM(O19:O21)</f>
-        <v>447.35250000000002</v>
+        <f t="shared" ref="O22:R22" si="14">SUM(O19:O21)</f>
+        <v>444.52699999999999</v>
       </c>
       <c r="P22" s="3">
+        <f t="shared" si="14"/>
+        <v>485.26799999999997</v>
+      </c>
+      <c r="Q22" s="3">
+        <f t="shared" si="14"/>
+        <v>443.01600000000008</v>
+      </c>
+      <c r="R22" s="3">
+        <f t="shared" si="14"/>
+        <v>456.79551750000007</v>
+      </c>
+      <c r="U22" s="3">
+        <f t="shared" ref="U22" si="15">SUM(U19:U21)</f>
+        <v>903.654</v>
+      </c>
+      <c r="V22" s="3">
+        <f t="shared" ref="V22:W22" si="16">SUM(V19:V21)</f>
+        <v>1281.3910000000001</v>
+      </c>
+      <c r="W22" s="3">
         <f t="shared" si="16"/>
-        <v>442.36079999999998</v>
-      </c>
-      <c r="Q22" s="3">
-        <f t="shared" si="16"/>
-        <v>443.01600000000008</v>
-      </c>
-      <c r="R22" s="3">
-        <f t="shared" si="16"/>
-        <v>456.79551750000007</v>
-      </c>
-      <c r="U22" s="3">
-        <f t="shared" ref="U22" si="17">SUM(U19:U21)</f>
-        <v>903.654</v>
-      </c>
-      <c r="V22" s="3">
-        <f t="shared" ref="V22:W22" si="18">SUM(V19:V21)</f>
-        <v>1281.3910000000001</v>
-      </c>
-      <c r="W22" s="3">
+        <v>1492.258</v>
+      </c>
+      <c r="X22" s="3">
+        <f t="shared" ref="X22:Y22" si="17">SUM(X19:X21)</f>
+        <v>1704.30935</v>
+      </c>
+      <c r="Y22" s="3">
+        <f t="shared" si="17"/>
+        <v>1829.6065175000001</v>
+      </c>
+      <c r="Z22" s="3">
+        <f t="shared" ref="Z22:AA22" si="18">SUM(Z19:Z21)</f>
+        <v>1921.0868433750002</v>
+      </c>
+      <c r="AA22" s="3">
         <f t="shared" si="18"/>
-        <v>1492.258</v>
-      </c>
-      <c r="X22" s="3">
-        <f t="shared" ref="X22:Y22" si="19">SUM(X19:X21)</f>
-        <v>1704.30935</v>
-      </c>
-      <c r="Y22" s="3">
-        <f t="shared" si="19"/>
-        <v>1789.5248175000004</v>
-      </c>
-      <c r="Z22" s="3">
-        <f t="shared" ref="Z22:AA22" si="20">SUM(Z19:Z21)</f>
-        <v>1879.0010583750002</v>
-      </c>
-      <c r="AA22" s="3">
-        <f t="shared" si="20"/>
-        <v>1972.9511112937507</v>
+        <v>2017.1411855437502</v>
       </c>
     </row>
     <row r="23" spans="2:27" x14ac:dyDescent="0.2">
@@ -2403,96 +2397,96 @@
         <v>36</v>
       </c>
       <c r="C23" s="3">
-        <f t="shared" ref="C23:N23" si="21">C18-C22</f>
+        <f t="shared" ref="C23:N23" si="19">C18-C22</f>
         <v>0</v>
       </c>
       <c r="D23" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="19"/>
         <v>-119.40599999999995</v>
       </c>
       <c r="E23" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="19"/>
         <v>-82.923000000000059</v>
       </c>
       <c r="F23" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="19"/>
         <v>-72.948999999999955</v>
       </c>
       <c r="G23" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="19"/>
         <v>-68.547000000000082</v>
       </c>
       <c r="H23" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="19"/>
         <v>-49.002999999999986</v>
       </c>
       <c r="I23" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="19"/>
         <v>-45.216000000000008</v>
       </c>
       <c r="J23" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="19"/>
         <v>-70.966000000000008</v>
       </c>
       <c r="K23" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="19"/>
         <v>-98.185999999999979</v>
       </c>
       <c r="L23" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="19"/>
         <v>-71.44</v>
       </c>
       <c r="M23" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="19"/>
         <v>-27.876000000000033</v>
       </c>
       <c r="N23" s="3">
-        <f t="shared" si="21"/>
+        <f t="shared" si="19"/>
         <v>-51.723350000000039</v>
       </c>
       <c r="O23" s="3">
-        <f t="shared" ref="O23:R23" si="22">O18-O22</f>
-        <v>-44.792500000000018</v>
+        <f t="shared" ref="O23:R23" si="20">O18-O22</f>
+        <v>-53.553999999999974</v>
       </c>
       <c r="P23" s="3">
+        <f t="shared" si="20"/>
+        <v>-65.293999999999926</v>
+      </c>
+      <c r="Q23" s="3">
+        <f t="shared" si="20"/>
+        <v>13.861479999999972</v>
+      </c>
+      <c r="R23" s="3">
+        <f t="shared" si="20"/>
+        <v>19.321962499999927</v>
+      </c>
+      <c r="U23" s="3">
+        <f t="shared" ref="U23" si="21">U18-U22</f>
+        <v>-289.36400000000003</v>
+      </c>
+      <c r="V23" s="3">
+        <f t="shared" ref="V23:W23" si="22">V18-V22</f>
+        <v>-346.6550000000002</v>
+      </c>
+      <c r="W23" s="3">
         <f t="shared" si="22"/>
-        <v>-20.560799999999972</v>
-      </c>
-      <c r="Q23" s="3">
-        <f t="shared" si="22"/>
-        <v>-1.9760000000000559</v>
-      </c>
-      <c r="R23" s="3">
-        <f t="shared" si="22"/>
-        <v>3.4844824999998991</v>
-      </c>
-      <c r="U23" s="3">
-        <f t="shared" ref="U23" si="23">U18-U22</f>
-        <v>-289.36400000000003</v>
-      </c>
-      <c r="V23" s="3">
-        <f t="shared" ref="V23:W23" si="24">V18-V22</f>
-        <v>-346.6550000000002</v>
-      </c>
-      <c r="W23" s="3">
+        <v>-233.7320000000002</v>
+      </c>
+      <c r="X23" s="3">
+        <f t="shared" ref="X23:Y23" si="23">X18-X22</f>
+        <v>-249.22534999999993</v>
+      </c>
+      <c r="Y23" s="3">
+        <f t="shared" si="23"/>
+        <v>-85.664557500000001</v>
+      </c>
+      <c r="Z23" s="3">
+        <f t="shared" ref="Z23:AA23" si="24">Z18-Z22</f>
+        <v>240.01115662500024</v>
+      </c>
+      <c r="AA23" s="3">
         <f t="shared" si="24"/>
-        <v>-233.7320000000002</v>
-      </c>
-      <c r="X23" s="3">
-        <f t="shared" ref="X23:Y23" si="25">X18-X22</f>
-        <v>-249.22534999999993</v>
-      </c>
-      <c r="Y23" s="3">
-        <f t="shared" si="25"/>
-        <v>-63.844817500000318</v>
-      </c>
-      <c r="Z23" s="3">
-        <f t="shared" ref="Z23:AA23" si="26">Z18-Z22</f>
-        <v>219.798941625</v>
-      </c>
-      <c r="AA23" s="3">
-        <f t="shared" si="26"/>
-        <v>545.60888870624922</v>
+        <v>576.17641445625009</v>
       </c>
     </row>
     <row r="24" spans="2:27" x14ac:dyDescent="0.2">
@@ -2539,20 +2533,20 @@
         <v>20.766999999999999</v>
       </c>
       <c r="O24" s="10">
-        <f>+N24</f>
-        <v>20.766999999999999</v>
+        <f>23.458-1.066-2.162</f>
+        <v>20.23</v>
       </c>
       <c r="P24" s="10">
-        <f>+O24</f>
-        <v>20.766999999999999</v>
+        <f>23.637-1.473</f>
+        <v>22.164000000000001</v>
       </c>
       <c r="Q24" s="10">
         <f>+P24</f>
-        <v>20.766999999999999</v>
+        <v>22.164000000000001</v>
       </c>
       <c r="R24" s="10">
         <f>+Q24</f>
-        <v>20.766999999999999</v>
+        <v>22.164000000000001</v>
       </c>
       <c r="U24" s="3">
         <f>0.926-11.316-3.135</f>
@@ -2563,24 +2557,24 @@
         <v>13.401</v>
       </c>
       <c r="W24" s="3">
-        <f t="shared" ref="W24" si="27">SUM(G24:J24)</f>
+        <f t="shared" ref="W24" si="25">SUM(G24:J24)</f>
         <v>70.215999999999994</v>
       </c>
       <c r="X24" s="10">
-        <f t="shared" ref="X24" si="28">SUM(K24:N24)</f>
+        <f t="shared" ref="X24" si="26">SUM(K24:N24)</f>
         <v>82.515999999999991</v>
       </c>
       <c r="Y24" s="10">
-        <f t="shared" ref="Y24:Y26" si="29">SUM(O24:R24)</f>
-        <v>83.067999999999998</v>
+        <f t="shared" ref="Y24:Y26" si="27">SUM(O24:R24)</f>
+        <v>86.722000000000008</v>
       </c>
       <c r="Z24" s="3">
         <f>+Y24</f>
-        <v>83.067999999999998</v>
+        <v>86.722000000000008</v>
       </c>
       <c r="AA24" s="3">
         <f>+Z24</f>
-        <v>83.067999999999998</v>
+        <v>86.722000000000008</v>
       </c>
     </row>
     <row r="25" spans="2:27" x14ac:dyDescent="0.2">
@@ -2588,35 +2582,35 @@
         <v>38</v>
       </c>
       <c r="C25" s="3">
-        <f t="shared" ref="C25:J25" si="30">+C23+C24</f>
+        <f t="shared" ref="C25:J25" si="28">+C23+C24</f>
         <v>0</v>
       </c>
       <c r="D25" s="3">
-        <f t="shared" si="30"/>
+        <f t="shared" si="28"/>
         <v>-120.37899999999995</v>
       </c>
       <c r="E25" s="3">
-        <f t="shared" si="30"/>
+        <f t="shared" si="28"/>
         <v>-79.806000000000054</v>
       </c>
       <c r="F25" s="3">
-        <f t="shared" si="30"/>
+        <f t="shared" si="28"/>
         <v>-61.483999999999952</v>
       </c>
       <c r="G25" s="3">
-        <f t="shared" si="30"/>
+        <f t="shared" si="28"/>
         <v>-51.759000000000086</v>
       </c>
       <c r="H25" s="3">
-        <f t="shared" si="30"/>
+        <f t="shared" si="28"/>
         <v>-34.008999999999986</v>
       </c>
       <c r="I25" s="3">
-        <f t="shared" si="30"/>
+        <f t="shared" si="28"/>
         <v>-25.662000000000006</v>
       </c>
       <c r="J25" s="3">
-        <f t="shared" si="30"/>
+        <f t="shared" si="28"/>
         <v>-52.086000000000013</v>
       </c>
       <c r="K25" s="3">
@@ -2636,48 +2630,48 @@
         <v>-30.95635000000004</v>
       </c>
       <c r="O25" s="3">
-        <f t="shared" ref="O25:R25" si="31">+O23+O24</f>
-        <v>-24.025500000000019</v>
+        <f t="shared" ref="O25:R25" si="29">+O23+O24</f>
+        <v>-33.32399999999997</v>
       </c>
       <c r="P25" s="3">
-        <f t="shared" si="31"/>
-        <v>0.20620000000002747</v>
+        <f t="shared" si="29"/>
+        <v>-43.129999999999924</v>
       </c>
       <c r="Q25" s="3">
-        <f t="shared" si="31"/>
-        <v>18.790999999999944</v>
+        <f t="shared" si="29"/>
+        <v>36.025479999999973</v>
       </c>
       <c r="R25" s="3">
-        <f t="shared" si="31"/>
-        <v>24.251482499999899</v>
+        <f t="shared" si="29"/>
+        <v>41.485962499999928</v>
       </c>
       <c r="U25" s="3">
-        <f t="shared" ref="U25:AA25" si="32">+U23+U24</f>
+        <f t="shared" ref="U25:AA25" si="30">+U23+U24</f>
         <v>-302.88900000000001</v>
       </c>
       <c r="V25" s="3">
-        <f t="shared" si="32"/>
+        <f t="shared" si="30"/>
         <v>-333.25400000000019</v>
       </c>
       <c r="W25" s="3">
-        <f t="shared" si="32"/>
+        <f t="shared" si="30"/>
         <v>-163.51600000000019</v>
       </c>
       <c r="X25" s="3">
-        <f t="shared" si="32"/>
+        <f t="shared" si="30"/>
         <v>-166.70934999999994</v>
       </c>
       <c r="Y25" s="3">
-        <f t="shared" si="32"/>
-        <v>19.22318249999968</v>
+        <f t="shared" si="30"/>
+        <v>1.0574425000000076</v>
       </c>
       <c r="Z25" s="3">
-        <f t="shared" si="32"/>
-        <v>302.86694162499998</v>
+        <f t="shared" si="30"/>
+        <v>326.73315662500022</v>
       </c>
       <c r="AA25" s="3">
-        <f t="shared" si="32"/>
-        <v>628.6768887062492</v>
+        <f t="shared" si="30"/>
+        <v>662.89841445625007</v>
       </c>
     </row>
     <row r="26" spans="2:27" x14ac:dyDescent="0.2">
@@ -2718,11 +2712,11 @@
       <c r="N26" s="12">
         <v>0</v>
       </c>
-      <c r="O26" s="12">
-        <v>0</v>
-      </c>
-      <c r="P26" s="12">
-        <v>0</v>
+      <c r="O26" s="26">
+        <v>4.3019999999999996</v>
+      </c>
+      <c r="P26" s="26">
+        <v>3.9279999999999999</v>
       </c>
       <c r="Q26" s="12">
         <v>0</v>
@@ -2737,24 +2731,24 @@
         <v>12.144</v>
       </c>
       <c r="W26" s="3">
-        <f t="shared" ref="W26" si="33">SUM(G26:J26)</f>
+        <f t="shared" ref="W26" si="31">SUM(G26:J26)</f>
         <v>13.084000000000001</v>
       </c>
       <c r="X26" s="10">
-        <f t="shared" ref="X26" si="34">SUM(K26:N26)</f>
+        <f t="shared" ref="X26" si="32">SUM(K26:N26)</f>
         <v>9.1449999999999996</v>
       </c>
       <c r="Y26" s="10">
-        <f t="shared" si="29"/>
-        <v>0</v>
+        <f t="shared" si="27"/>
+        <v>8.23</v>
       </c>
       <c r="Z26" s="3">
         <f>+Z25*0.1</f>
-        <v>30.286694162499998</v>
+        <v>32.673315662500023</v>
       </c>
       <c r="AA26" s="3">
         <f>+AA25*0.2</f>
-        <v>125.73537774124985</v>
+        <v>132.57968289125003</v>
       </c>
     </row>
     <row r="27" spans="2:27" x14ac:dyDescent="0.2">
@@ -2762,35 +2756,35 @@
         <v>8</v>
       </c>
       <c r="C27" s="3">
-        <f t="shared" ref="C27:J27" si="35">+C25-C26</f>
+        <f t="shared" ref="C27:J27" si="33">+C25-C26</f>
         <v>0</v>
       </c>
       <c r="D27" s="3">
-        <f t="shared" si="35"/>
+        <f t="shared" si="33"/>
         <v>-123.42799999999995</v>
       </c>
       <c r="E27" s="3">
-        <f t="shared" si="35"/>
+        <f t="shared" si="33"/>
         <v>-84.841000000000051</v>
       </c>
       <c r="F27" s="3">
-        <f t="shared" si="35"/>
+        <f t="shared" si="33"/>
         <v>-64.397999999999954</v>
       </c>
       <c r="G27" s="3">
-        <f t="shared" si="35"/>
+        <f t="shared" si="33"/>
         <v>-54.246000000000087</v>
       </c>
       <c r="H27" s="3">
-        <f t="shared" si="35"/>
+        <f t="shared" si="33"/>
         <v>-37.596999999999987</v>
       </c>
       <c r="I27" s="3">
-        <f t="shared" si="35"/>
+        <f t="shared" si="33"/>
         <v>-29.297000000000004</v>
       </c>
       <c r="J27" s="3">
-        <f t="shared" si="35"/>
+        <f t="shared" si="33"/>
         <v>-55.460000000000015</v>
       </c>
       <c r="K27" s="3">
@@ -2810,48 +2804,48 @@
         <v>-30.95635000000004</v>
       </c>
       <c r="O27" s="3">
-        <f t="shared" ref="O27:R27" si="36">+O25-O26</f>
-        <v>-24.025500000000019</v>
+        <f t="shared" ref="O27:R27" si="34">+O25-O26</f>
+        <v>-37.625999999999969</v>
       </c>
       <c r="P27" s="3">
-        <f t="shared" si="36"/>
-        <v>0.20620000000002747</v>
+        <f t="shared" si="34"/>
+        <v>-47.057999999999922</v>
       </c>
       <c r="Q27" s="3">
-        <f t="shared" si="36"/>
-        <v>18.790999999999944</v>
+        <f t="shared" si="34"/>
+        <v>36.025479999999973</v>
       </c>
       <c r="R27" s="3">
-        <f t="shared" si="36"/>
-        <v>24.251482499999899</v>
+        <f t="shared" si="34"/>
+        <v>41.485962499999928</v>
       </c>
       <c r="U27" s="3">
-        <f t="shared" ref="U27:AA27" si="37">+U25-U26</f>
+        <f t="shared" ref="U27:AA27" si="35">+U25-U26</f>
         <v>-306.86599999999999</v>
       </c>
       <c r="V27" s="3">
-        <f t="shared" si="37"/>
+        <f t="shared" si="35"/>
         <v>-345.3980000000002</v>
       </c>
       <c r="W27" s="3">
-        <f t="shared" si="37"/>
+        <f t="shared" si="35"/>
         <v>-176.60000000000019</v>
       </c>
       <c r="X27" s="3">
-        <f t="shared" si="37"/>
+        <f t="shared" si="35"/>
         <v>-175.85434999999995</v>
       </c>
       <c r="Y27" s="3">
-        <f t="shared" si="37"/>
-        <v>19.22318249999968</v>
+        <f t="shared" si="35"/>
+        <v>-7.1725574999999928</v>
       </c>
       <c r="Z27" s="3">
-        <f t="shared" si="37"/>
-        <v>272.58024746249998</v>
+        <f t="shared" si="35"/>
+        <v>294.05984096250018</v>
       </c>
       <c r="AA27" s="3">
-        <f t="shared" si="37"/>
-        <v>502.94151096499934</v>
+        <f t="shared" si="35"/>
+        <v>530.31873156500001</v>
       </c>
     </row>
     <row r="28" spans="2:27" x14ac:dyDescent="0.2">
@@ -2859,35 +2853,35 @@
         <v>40</v>
       </c>
       <c r="C28" s="7" t="e">
-        <f t="shared" ref="C28:J28" si="38">C27/C29</f>
+        <f t="shared" ref="C28:J28" si="36">C27/C29</f>
         <v>#DIV/0!</v>
       </c>
       <c r="D28" s="7">
-        <f t="shared" si="38"/>
+        <f t="shared" si="36"/>
         <v>-1.8062335280774275</v>
       </c>
       <c r="E28" s="7">
-        <f t="shared" si="38"/>
+        <f t="shared" si="36"/>
         <v>-1.2310638914773968</v>
       </c>
       <c r="F28" s="7">
-        <f t="shared" si="38"/>
+        <f t="shared" si="36"/>
         <v>-0.92625357140093434</v>
       </c>
       <c r="G28" s="7">
-        <f t="shared" si="38"/>
+        <f t="shared" si="36"/>
         <v>-0.77298280464511981</v>
       </c>
       <c r="H28" s="7">
-        <f t="shared" si="38"/>
+        <f t="shared" si="36"/>
         <v>-0.53047574476307036</v>
       </c>
       <c r="I28" s="7">
-        <f t="shared" si="38"/>
+        <f t="shared" si="36"/>
         <v>-0.40940456377438567</v>
       </c>
       <c r="J28" s="7">
-        <f t="shared" si="38"/>
+        <f t="shared" si="36"/>
         <v>-0.76655837267370075</v>
       </c>
       <c r="K28" s="7">
@@ -2907,48 +2901,48 @@
         <v>-0.41821267224919473</v>
       </c>
       <c r="O28" s="7">
-        <f t="shared" ref="O28:R28" si="39">O27/O29</f>
-        <v>-0.32457859395965682</v>
+        <f t="shared" ref="O28:R28" si="37">O27/O29</f>
+        <v>-0.46416997843915236</v>
       </c>
       <c r="P28" s="7">
-        <f t="shared" si="39"/>
-        <v>2.5456790123460182E-3</v>
+        <f t="shared" si="37"/>
+        <v>-0.58040405535410244</v>
       </c>
       <c r="Q28" s="7">
-        <f t="shared" si="39"/>
-        <v>0.23198765432098695</v>
+        <f t="shared" si="37"/>
+        <v>0.4443311379165738</v>
       </c>
       <c r="R28" s="7">
-        <f t="shared" si="39"/>
-        <v>0.29940101851851725</v>
+        <f t="shared" si="37"/>
+        <v>0.51167964799328947</v>
       </c>
       <c r="U28" s="7">
-        <f t="shared" ref="U28:AA28" si="40">U27/U29</f>
+        <f t="shared" ref="U28:AA28" si="38">U27/U29</f>
         <v>-4.7529676115582671</v>
       </c>
       <c r="V28" s="7">
-        <f t="shared" si="40"/>
+        <f t="shared" si="38"/>
         <v>-5.0328824418661222</v>
       </c>
       <c r="W28" s="7">
-        <f t="shared" si="40"/>
+        <f t="shared" si="38"/>
         <v>-2.478935809701309</v>
       </c>
       <c r="X28" s="7">
-        <f t="shared" si="40"/>
+        <f t="shared" si="38"/>
         <v>-2.171041358024691</v>
       </c>
       <c r="Y28" s="7">
-        <f t="shared" si="40"/>
-        <v>0.2373232407407368</v>
+        <f t="shared" si="38"/>
+        <v>-8.85500925925925E-2</v>
       </c>
       <c r="Z28" s="7">
-        <f t="shared" si="40"/>
-        <v>3.3651882402777775</v>
+        <f t="shared" si="38"/>
+        <v>3.6303684069444464</v>
       </c>
       <c r="AA28" s="7">
-        <f t="shared" si="40"/>
-        <v>6.2091544563580161</v>
+        <f t="shared" si="38"/>
+        <v>6.5471448341358025</v>
       </c>
     </row>
     <row r="29" spans="2:27" x14ac:dyDescent="0.2">
@@ -2991,19 +2985,18 @@
         <v>74.020593000000005</v>
       </c>
       <c r="O29" s="10">
-        <f>+N29</f>
-        <v>74.020593000000005</v>
+        <v>81.060822000000002</v>
       </c>
       <c r="P29" s="10">
-        <v>81</v>
+        <v>81.078000000000003</v>
       </c>
       <c r="Q29" s="10">
-        <f t="shared" ref="P29:R29" si="41">+P29</f>
-        <v>81</v>
+        <f t="shared" ref="Q29:R29" si="39">+P29</f>
+        <v>81.078000000000003</v>
       </c>
       <c r="R29" s="10">
-        <f t="shared" si="41"/>
-        <v>81</v>
+        <f t="shared" si="39"/>
+        <v>81.078000000000003</v>
       </c>
       <c r="U29" s="3">
         <v>64.563032000000007</v>
@@ -3037,71 +3030,71 @@
       <c r="F31" s="5"/>
       <c r="G31" s="5"/>
       <c r="H31" s="5">
-        <f t="shared" ref="H31:R31" si="42">H16/D16-1</f>
+        <f t="shared" ref="H31:R31" si="40">H16/D16-1</f>
         <v>0.39188825245014303</v>
       </c>
       <c r="I31" s="5">
-        <f t="shared" si="42"/>
+        <f t="shared" si="40"/>
         <v>0.29769409000032976</v>
       </c>
       <c r="J31" s="5">
-        <f t="shared" si="42"/>
+        <f t="shared" si="40"/>
         <v>0.26760805065981752</v>
       </c>
       <c r="K31" s="5">
-        <f t="shared" si="42"/>
+        <f t="shared" si="40"/>
         <v>0.22341968067774531</v>
       </c>
       <c r="L31" s="5">
-        <f t="shared" si="42"/>
+        <f t="shared" si="40"/>
         <v>0.12817166952578041</v>
       </c>
       <c r="M31" s="5">
-        <f t="shared" si="42"/>
+        <f t="shared" si="40"/>
         <v>0.22275013974287305</v>
       </c>
       <c r="N31" s="5">
-        <f t="shared" si="42"/>
+        <f t="shared" si="40"/>
         <v>0.13099942795009634</v>
       </c>
       <c r="O31" s="5">
-        <f t="shared" si="42"/>
-        <v>0.20738368389629813</v>
+        <f t="shared" si="40"/>
+        <v>0.21851203277691589</v>
       </c>
       <c r="P31" s="5">
-        <f t="shared" si="42"/>
-        <v>0.19219675847976103</v>
+        <f t="shared" si="40"/>
+        <v>0.23696060940078523</v>
       </c>
       <c r="Q31" s="5">
-        <f t="shared" si="42"/>
-        <v>0.12585596221959849</v>
+        <f t="shared" si="40"/>
+        <v>0.16628476977567885</v>
       </c>
       <c r="R31" s="5">
-        <f t="shared" si="42"/>
-        <v>0.20077220077220082</v>
+        <f t="shared" si="40"/>
+        <v>0.2420888030888031</v>
       </c>
       <c r="V31" s="19">
-        <f t="shared" ref="V31:AA31" si="43">+V16/U16-1</f>
+        <f t="shared" ref="V31:AA31" si="41">+V16/U16-1</f>
         <v>0.46951985735572488</v>
       </c>
       <c r="W31" s="19">
-        <f t="shared" si="43"/>
+        <f t="shared" si="41"/>
         <v>0.31071539827419703</v>
       </c>
       <c r="X31" s="19">
-        <f t="shared" si="43"/>
+        <f t="shared" si="41"/>
         <v>0.17411294400333688</v>
       </c>
       <c r="Y31" s="19">
-        <f t="shared" si="43"/>
-        <v>0.18013506777426613</v>
+        <f t="shared" si="41"/>
+        <v>0.21516463440862954</v>
       </c>
       <c r="Z31" s="19">
-        <f t="shared" si="43"/>
+        <f t="shared" si="41"/>
         <v>0.19999999999999996</v>
       </c>
       <c r="AA31" s="19">
-        <f t="shared" si="43"/>
+        <f t="shared" si="41"/>
         <v>0.19999999999999996</v>
       </c>
     </row>
@@ -3110,91 +3103,91 @@
         <v>90</v>
       </c>
       <c r="D32" s="19">
-        <f t="shared" ref="D32:F32" si="44">+D18/D16</f>
+        <f t="shared" ref="D32:F32" si="42">+D18/D16</f>
         <v>0.69241178170734918</v>
       </c>
       <c r="E32" s="19">
+        <f t="shared" si="42"/>
+        <v>0.71928625596110563</v>
+      </c>
+      <c r="F32" s="19">
+        <f t="shared" si="42"/>
+        <v>0.75323266318306625</v>
+      </c>
+      <c r="G32" s="19">
+        <f t="shared" ref="G32:L32" si="43">+G18/G16</f>
+        <v>0.73539426523297491</v>
+      </c>
+      <c r="H32" s="19">
+        <f t="shared" si="43"/>
+        <v>0.75144115849557924</v>
+      </c>
+      <c r="I32" s="19">
+        <f t="shared" si="43"/>
+        <v>0.75271747917715703</v>
+      </c>
+      <c r="J32" s="19">
+        <f t="shared" si="43"/>
+        <v>0.74969323278064282</v>
+      </c>
+      <c r="K32" s="19">
+        <f t="shared" si="43"/>
+        <v>0.72767949289885281</v>
+      </c>
+      <c r="L32" s="19">
+        <f t="shared" si="43"/>
+        <v>0.73174945462227237</v>
+      </c>
+      <c r="M32" s="19">
+        <f t="shared" ref="M32:R32" si="44">+M18/M16</f>
+        <v>0.74435702479338839</v>
+      </c>
+      <c r="N32" s="19">
         <f t="shared" si="44"/>
-        <v>0.71928625596110563</v>
-      </c>
-      <c r="F32" s="19">
+        <v>0.74</v>
+      </c>
+      <c r="O32" s="19">
         <f t="shared" si="44"/>
-        <v>0.75323266318306625</v>
-      </c>
-      <c r="G32" s="19">
-        <f t="shared" ref="G32:L32" si="45">+G18/G16</f>
-        <v>0.73539426523297491</v>
-      </c>
-      <c r="H32" s="19">
+        <v>0.71213666682452548</v>
+      </c>
+      <c r="P32" s="19">
+        <f t="shared" si="44"/>
+        <v>0.71013287070385289</v>
+      </c>
+      <c r="Q32" s="19">
+        <f t="shared" si="44"/>
+        <v>0.74</v>
+      </c>
+      <c r="R32" s="19">
+        <f t="shared" si="44"/>
+        <v>0.74</v>
+      </c>
+      <c r="U32" s="19">
+        <f t="shared" ref="U32:AA32" si="45">+U18/U16</f>
+        <v>0.703024324144924</v>
+      </c>
+      <c r="V32" s="19">
         <f t="shared" si="45"/>
-        <v>0.75144115849557924</v>
-      </c>
-      <c r="I32" s="19">
+        <v>0.7279648609077598</v>
+      </c>
+      <c r="W32" s="19">
         <f t="shared" si="45"/>
-        <v>0.75271747917715703</v>
-      </c>
-      <c r="J32" s="19">
+        <v>0.74778239714416594</v>
+      </c>
+      <c r="X32" s="19">
         <f t="shared" si="45"/>
-        <v>0.74969323278064282</v>
-      </c>
-      <c r="K32" s="19">
+        <v>0.73636177313775752</v>
+      </c>
+      <c r="Y32" s="19">
         <f t="shared" si="45"/>
-        <v>0.72767949289885281</v>
-      </c>
-      <c r="L32" s="19">
+        <v>0.72627329440867561</v>
+      </c>
+      <c r="Z32" s="19">
         <f t="shared" si="45"/>
-        <v>0.73174945462227237</v>
-      </c>
-      <c r="M32" s="19">
-        <f t="shared" ref="M32:R32" si="46">+M18/M16</f>
-        <v>0.74435702479338839</v>
-      </c>
-      <c r="N32" s="19">
-        <f t="shared" si="46"/>
-        <v>0.74</v>
-      </c>
-      <c r="O32" s="19">
-        <f t="shared" si="46"/>
-        <v>0.74</v>
-      </c>
-      <c r="P32" s="19">
-        <f t="shared" si="46"/>
-        <v>0.74</v>
-      </c>
-      <c r="Q32" s="19">
-        <f t="shared" si="46"/>
-        <v>0.74</v>
-      </c>
-      <c r="R32" s="19">
-        <f t="shared" si="46"/>
-        <v>0.74</v>
-      </c>
-      <c r="U32" s="19">
-        <f t="shared" ref="U32:AA32" si="47">+U18/U16</f>
-        <v>0.703024324144924</v>
-      </c>
-      <c r="V32" s="19">
-        <f t="shared" si="47"/>
-        <v>0.7279648609077598</v>
-      </c>
-      <c r="W32" s="19">
-        <f t="shared" si="47"/>
-        <v>0.74778239714416594</v>
-      </c>
-      <c r="X32" s="19">
-        <f t="shared" si="47"/>
-        <v>0.73636177313775752</v>
-      </c>
-      <c r="Y32" s="19">
-        <f t="shared" si="47"/>
-        <v>0.74</v>
-      </c>
-      <c r="Z32" s="19">
-        <f t="shared" si="47"/>
         <v>0.75</v>
       </c>
       <c r="AA32" s="19">
-        <f t="shared" si="47"/>
+        <f t="shared" si="45"/>
         <v>0.75</v>
       </c>
     </row>
@@ -3351,7 +3344,7 @@
       </c>
       <c r="AC39" s="21">
         <f>NPV(AC38,U16:BY16)</f>
-        <v>47391.850417467293</v>
+        <v>48669.102445567631</v>
       </c>
     </row>
     <row r="40" spans="2:33" x14ac:dyDescent="0.2">
@@ -3414,7 +3407,7 @@
       </c>
       <c r="AC41" s="21">
         <f>AC39/AC40</f>
-        <v>585.08457305515174</v>
+        <v>600.85311661194601</v>
       </c>
     </row>
     <row r="42" spans="2:33" ht="15.75" x14ac:dyDescent="0.25">
@@ -3444,7 +3437,7 @@
       </c>
       <c r="AC42" s="23">
         <f>(AC41-Main!J2)/Main!J2</f>
-        <v>0.84884210660162984</v>
+        <v>0.89867002658138795</v>
       </c>
     </row>
     <row r="43" spans="2:33" x14ac:dyDescent="0.2">
@@ -3499,14 +3492,14 @@
     </row>
     <row r="45" spans="2:33" ht="85.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="L45" s="3"/>
-      <c r="AB45" s="24" t="s">
+      <c r="AB45" s="25" t="s">
         <v>115</v>
       </c>
-      <c r="AC45" s="24"/>
-      <c r="AD45" s="24"/>
-      <c r="AE45" s="25"/>
-      <c r="AF45" s="25"/>
-      <c r="AG45" s="25"/>
+      <c r="AC45" s="25"/>
+      <c r="AD45" s="25"/>
+      <c r="AE45" s="24"/>
+      <c r="AF45" s="24"/>
+      <c r="AG45" s="24"/>
     </row>
     <row r="46" spans="2:33" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
@@ -3530,12 +3523,12 @@
       <c r="M46" s="10">
         <v>11.444000000000001</v>
       </c>
-      <c r="AB46" s="25"/>
-      <c r="AC46" s="25"/>
-      <c r="AD46" s="25"/>
-      <c r="AE46" s="25"/>
-      <c r="AF46" s="25"/>
-      <c r="AG46" s="25"/>
+      <c r="AB46" s="24"/>
+      <c r="AC46" s="24"/>
+      <c r="AD46" s="24"/>
+      <c r="AE46" s="24"/>
+      <c r="AF46" s="24"/>
+      <c r="AG46" s="24"/>
     </row>
     <row r="47" spans="2:33" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
@@ -3559,12 +3552,12 @@
       <c r="M47" s="10">
         <v>120.598</v>
       </c>
-      <c r="AB47" s="25"/>
-      <c r="AC47" s="25"/>
-      <c r="AD47" s="25"/>
-      <c r="AE47" s="25"/>
-      <c r="AF47" s="25"/>
-      <c r="AG47" s="25"/>
+      <c r="AB47" s="24"/>
+      <c r="AC47" s="24"/>
+      <c r="AD47" s="24"/>
+      <c r="AE47" s="24"/>
+      <c r="AF47" s="24"/>
+      <c r="AG47" s="24"/>
     </row>
     <row r="48" spans="2:33" x14ac:dyDescent="0.2">
       <c r="B48" s="1" t="s">
@@ -3592,12 +3585,12 @@
         <f>10.787+27.639</f>
         <v>38.426000000000002</v>
       </c>
-      <c r="AB48" s="25"/>
-      <c r="AC48" s="25"/>
-      <c r="AD48" s="25"/>
-      <c r="AE48" s="25"/>
-      <c r="AF48" s="25"/>
-      <c r="AG48" s="25"/>
+      <c r="AB48" s="24"/>
+      <c r="AC48" s="24"/>
+      <c r="AD48" s="24"/>
+      <c r="AE48" s="24"/>
+      <c r="AF48" s="24"/>
+      <c r="AG48" s="24"/>
     </row>
     <row r="49" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B49" s="1" t="s">
@@ -3791,15 +3784,15 @@
         <v>-9.7760000000000336</v>
       </c>
       <c r="U57" s="10">
-        <f t="shared" ref="U57:W57" si="48">+U27</f>
+        <f t="shared" ref="U57:W57" si="46">+U27</f>
         <v>-306.86599999999999</v>
       </c>
       <c r="V57" s="10">
-        <f t="shared" si="48"/>
+        <f t="shared" si="46"/>
         <v>-345.3980000000002</v>
       </c>
       <c r="W57" s="10">
-        <f t="shared" si="48"/>
+        <f t="shared" si="46"/>
         <v>-176.60000000000019</v>
       </c>
       <c r="X57" s="10">
@@ -3808,7 +3801,7 @@
       </c>
       <c r="Y57" s="10">
         <f>+Y27</f>
-        <v>19.22318249999968</v>
+        <v>-7.1725574999999928</v>
       </c>
     </row>
     <row r="58" spans="2:25" x14ac:dyDescent="0.2">
@@ -4322,15 +4315,15 @@
         <v>35.457000000000001</v>
       </c>
       <c r="U85" s="3">
-        <f t="shared" ref="U85:W85" si="49">+U65+U67</f>
+        <f t="shared" ref="U85:W85" si="47">+U65+U67</f>
         <v>-1.0920000000000236</v>
       </c>
       <c r="V85" s="3">
-        <f t="shared" si="49"/>
+        <f t="shared" si="47"/>
         <v>-20.21399999999997</v>
       </c>
       <c r="W85" s="3">
-        <f t="shared" si="49"/>
+        <f t="shared" si="47"/>
         <v>113.405</v>
       </c>
     </row>

</xml_diff>